<commit_message>
Update case timing workbook
</commit_message>
<xml_diff>
--- a/times .xlsx
+++ b/times .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Room_8_Data\Scalpel_Raz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{065A9DE0-73DA-4562-88C0-E8D33D2F5023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDEB2F3-8FDF-4D85-A515-D5E7FDCAA80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="196">
   <si>
     <t>date</t>
   </si>
@@ -598,6 +598,21 @@
   </si>
   <si>
     <t>no patient + ventilation</t>
+  </si>
+  <si>
+    <t>dead time</t>
+  </si>
+  <si>
+    <t>??</t>
+  </si>
+  <si>
+    <t>not a case</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 07:01:03</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> start</t>
   </si>
 </sst>
 </file>
@@ -1082,10 +1097,10 @@
         <v>23</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1115,6 +1130,9 @@
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="B13" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D13" s="4"/>
     </row>
     <row r="14" spans="1:8">
@@ -1186,15 +1204,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:8">
       <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>7</v>
+      <c r="B17" s="3">
+        <v>9.525462962962963E-3</v>
+      </c>
+      <c r="C17" s="3">
+        <v>4.431712962962963E-2</v>
+      </c>
+      <c r="D17" s="3">
+        <v>7.9085648148148155E-2</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0.14275462962962962</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>7</v>
@@ -1203,249 +1227,513 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:8">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="B19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="B20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="3">
+        <v>7.5289351851851857E-2</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="B21" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="B22" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="B23" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="3">
+        <v>4.7546296296296295E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="26" spans="1:7">
+      <c r="D25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="3">
+        <v>1.8576388888888889E-2</v>
+      </c>
+      <c r="F25" s="3">
+        <v>3.1805555555555552E-2</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H25" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="27" spans="1:7">
+      <c r="B26" s="3">
+        <v>1.8981481481481482E-3</v>
+      </c>
+      <c r="C26" s="3">
+        <v>7.3530092592592591E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="B27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="29" spans="1:7">
+      <c r="B28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="3">
+        <v>0.12725694444444444</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="B29" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0.25537037037037036</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="B30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="3">
+        <v>5.8252314814814812E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="32" spans="1:7">
+      <c r="B31" s="3">
+        <v>4.2013888888888891E-3</v>
+      </c>
+      <c r="C31" s="3">
+        <v>8.5289351851851852E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="33" spans="1:1">
+      <c r="B32" s="3">
+        <v>8.8078703703703704E-3</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="34" spans="1:1">
+      <c r="B33" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="35" spans="1:1">
+      <c r="B34" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="36" spans="1:1">
+      <c r="B35" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="37" spans="1:1">
+      <c r="B36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="38" spans="1:1">
+      <c r="B37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" s="2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="39" spans="1:1">
+      <c r="B38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" s="3">
+        <v>7.6284722222222226E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="40" spans="1:1">
+      <c r="B39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="41" spans="1:1">
+      <c r="B40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="3">
+        <v>8.7696759259259266E-2</v>
+      </c>
+      <c r="D40" s="3">
+        <v>0.1218287037037037</v>
+      </c>
+      <c r="E40" s="3">
+        <v>0.18619212962962964</v>
+      </c>
+      <c r="F40" s="3">
+        <v>0.22163194444444445</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="42" spans="1:1">
+      <c r="B41" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="43" spans="1:1">
+      <c r="B42" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" s="2" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="44" spans="1:1">
+      <c r="B43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="45" spans="1:1">
+      <c r="B44" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="46" spans="1:1">
+      <c r="B45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" s="3">
+        <v>0.18371527777777777</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="47" spans="1:1">
+      <c r="B46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" s="3">
+        <v>0.12155092592592592</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" s="2" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="48" spans="1:1">
+      <c r="B47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" s="2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="49" spans="1:1">
+      <c r="B48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" s="3">
+        <v>5.5069444444444442E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" s="2" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="50" spans="1:1">
+      <c r="B49" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" s="2" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="51" spans="1:1">
+      <c r="B50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="52" spans="1:1">
+      <c r="B51" s="3">
+        <v>1.1238425925925926E-2</v>
+      </c>
+      <c r="C51" s="3">
+        <v>0.12010416666666666</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="53" spans="1:1">
+      <c r="B52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" s="3">
+        <v>5.6678240740740737E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" s="2" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="54" spans="1:1">
+      <c r="B53" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C53" s="3">
+        <v>3.0393518518518518E-2</v>
+      </c>
+      <c r="D53" s="3">
+        <v>7.2951388888888885E-2</v>
+      </c>
+      <c r="E53" s="3">
+        <v>0.19527777777777777</v>
+      </c>
+      <c r="H53" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="55" spans="1:1">
+      <c r="B54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="56" spans="1:1">
+      <c r="B55" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C55" s="3">
+        <v>9.6782407407407414E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="57" spans="1:1">
+      <c r="B56" s="3">
+        <v>5.0694444444444441E-3</v>
+      </c>
+      <c r="C56" s="3">
+        <v>0.12431712962962962</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="58" spans="1:1">
+      <c r="B57" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C57" s="3">
+        <v>0.19346064814814815</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="59" spans="1:1">
+      <c r="B58" s="3">
+        <v>1.480324074074074E-2</v>
+      </c>
+      <c r="C58" s="3">
+        <v>7.7777777777777779E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="60" spans="1:1">
+      <c r="B59" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" s="3">
+        <v>0.11229166666666666</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
       <c r="A60" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="61" spans="1:1">
+      <c r="B60" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="3">
+        <v>0.16875000000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
       <c r="A61" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="62" spans="1:1">
+    <row r="62" spans="1:8">
       <c r="A62" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="63" spans="1:1">
+    <row r="63" spans="1:8">
       <c r="A63" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="64" spans="1:1">
+    <row r="64" spans="1:8">
       <c r="A64" s="2" t="s">
         <v>76</v>
       </c>

</xml_diff>

<commit_message>
on lab- update times .xlsx
</commit_message>
<xml_diff>
--- a/times .xlsx
+++ b/times .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Room_8_Data\Scalpel_Raz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{065A9DE0-73DA-4562-88C0-E8D33D2F5023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDEB2F3-8FDF-4D85-A515-D5E7FDCAA80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="196">
   <si>
     <t>date</t>
   </si>
@@ -598,6 +598,21 @@
   </si>
   <si>
     <t>no patient + ventilation</t>
+  </si>
+  <si>
+    <t>dead time</t>
+  </si>
+  <si>
+    <t>??</t>
+  </si>
+  <si>
+    <t>not a case</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 07:01:03</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> start</t>
   </si>
 </sst>
 </file>
@@ -1082,10 +1097,10 @@
         <v>23</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1115,6 +1130,9 @@
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="B13" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="D13" s="4"/>
     </row>
     <row r="14" spans="1:8">
@@ -1186,15 +1204,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:8">
       <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>7</v>
+      <c r="B17" s="3">
+        <v>9.525462962962963E-3</v>
+      </c>
+      <c r="C17" s="3">
+        <v>4.431712962962963E-2</v>
+      </c>
+      <c r="D17" s="3">
+        <v>7.9085648148148155E-2</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0.14275462962962962</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>7</v>
@@ -1203,249 +1227,513 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:8">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="B19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="B20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="3">
+        <v>7.5289351851851857E-2</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="B21" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="B22" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="B23" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="3">
+        <v>4.7546296296296295E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="26" spans="1:7">
+      <c r="D25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="3">
+        <v>1.8576388888888889E-2</v>
+      </c>
+      <c r="F25" s="3">
+        <v>3.1805555555555552E-2</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H25" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="27" spans="1:7">
+      <c r="B26" s="3">
+        <v>1.8981481481481482E-3</v>
+      </c>
+      <c r="C26" s="3">
+        <v>7.3530092592592591E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="B27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="29" spans="1:7">
+      <c r="B28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="3">
+        <v>0.12725694444444444</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="B29" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0.25537037037037036</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="B30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="3">
+        <v>5.8252314814814812E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="32" spans="1:7">
+      <c r="B31" s="3">
+        <v>4.2013888888888891E-3</v>
+      </c>
+      <c r="C31" s="3">
+        <v>8.5289351851851852E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="33" spans="1:1">
+      <c r="B32" s="3">
+        <v>8.8078703703703704E-3</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="34" spans="1:1">
+      <c r="B33" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="35" spans="1:1">
+      <c r="B34" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="36" spans="1:1">
+      <c r="B35" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="37" spans="1:1">
+      <c r="B36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="38" spans="1:1">
+      <c r="B37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" s="2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="39" spans="1:1">
+      <c r="B38" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" s="3">
+        <v>7.6284722222222226E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="40" spans="1:1">
+      <c r="B39" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="41" spans="1:1">
+      <c r="B40" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="3">
+        <v>8.7696759259259266E-2</v>
+      </c>
+      <c r="D40" s="3">
+        <v>0.1218287037037037</v>
+      </c>
+      <c r="E40" s="3">
+        <v>0.18619212962962964</v>
+      </c>
+      <c r="F40" s="3">
+        <v>0.22163194444444445</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="42" spans="1:1">
+      <c r="B41" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="43" spans="1:1">
+      <c r="B42" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" s="2" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="44" spans="1:1">
+      <c r="B43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="45" spans="1:1">
+      <c r="B44" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="46" spans="1:1">
+      <c r="B45" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" s="3">
+        <v>0.18371527777777777</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="47" spans="1:1">
+      <c r="B46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" s="3">
+        <v>0.12155092592592592</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" s="2" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="48" spans="1:1">
+      <c r="B47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" s="2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="49" spans="1:1">
+      <c r="B48" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" s="3">
+        <v>5.5069444444444442E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" s="2" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="50" spans="1:1">
+      <c r="B49" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" s="2" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="51" spans="1:1">
+      <c r="B50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="52" spans="1:1">
+      <c r="B51" s="3">
+        <v>1.1238425925925926E-2</v>
+      </c>
+      <c r="C51" s="3">
+        <v>0.12010416666666666</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="53" spans="1:1">
+      <c r="B52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" s="3">
+        <v>5.6678240740740737E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" s="2" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="54" spans="1:1">
+      <c r="B53" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C53" s="3">
+        <v>3.0393518518518518E-2</v>
+      </c>
+      <c r="D53" s="3">
+        <v>7.2951388888888885E-2</v>
+      </c>
+      <c r="E53" s="3">
+        <v>0.19527777777777777</v>
+      </c>
+      <c r="H53" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="55" spans="1:1">
+      <c r="B54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="56" spans="1:1">
+      <c r="B55" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C55" s="3">
+        <v>9.6782407407407414E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="57" spans="1:1">
+      <c r="B56" s="3">
+        <v>5.0694444444444441E-3</v>
+      </c>
+      <c r="C56" s="3">
+        <v>0.12431712962962962</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="58" spans="1:1">
+      <c r="B57" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C57" s="3">
+        <v>0.19346064814814815</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="59" spans="1:1">
+      <c r="B58" s="3">
+        <v>1.480324074074074E-2</v>
+      </c>
+      <c r="C58" s="3">
+        <v>7.7777777777777779E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="60" spans="1:1">
+      <c r="B59" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" s="3">
+        <v>0.11229166666666666</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
       <c r="A60" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="61" spans="1:1">
+      <c r="B60" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="3">
+        <v>0.16875000000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
       <c r="A61" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="62" spans="1:1">
+    <row r="62" spans="1:8">
       <c r="A62" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="63" spans="1:1">
+    <row r="63" spans="1:8">
       <c r="A63" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="64" spans="1:1">
+    <row r="64" spans="1:8">
       <c r="A64" s="2" t="s">
         <v>76</v>
       </c>

</xml_diff>

<commit_message>
Finalize case timing workbook updates
</commit_message>
<xml_diff>
--- a/times .xlsx
+++ b/times .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Room_8_Data\Scalpel_Raz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDEB2F3-8FDF-4D85-A515-D5E7FDCAA80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6755F6-9E17-48AE-95AF-D7B8A2C65CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="201">
   <si>
     <t>date</t>
   </si>
@@ -63,9 +63,6 @@
     <t>?</t>
   </si>
   <si>
-    <t>prbably end</t>
-  </si>
-  <si>
     <t>v</t>
   </si>
   <si>
@@ -613,6 +610,24 @@
   </si>
   <si>
     <t xml:space="preserve"> start</t>
+  </si>
+  <si>
+    <t>very long</t>
+  </si>
+  <si>
+    <t>14hrs</t>
+  </si>
+  <si>
+    <t>50hr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  01:13:07</t>
+  </si>
+  <si>
+    <t>19hr</t>
+  </si>
+  <si>
+    <t>Foramt problem. Export again</t>
   </si>
 </sst>
 </file>
@@ -985,8 +1000,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="45.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="19.125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="39.5" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.75" style="2" customWidth="1"/>
     <col min="6" max="6" width="16.5" style="2" bestFit="1" customWidth="1"/>
@@ -1019,15 +1033,15 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>7</v>
@@ -1035,7 +1049,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>7</v>
@@ -1043,26 +1057,26 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
@@ -1070,7 +1084,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>7</v>
@@ -1078,23 +1092,23 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>9</v>
@@ -1105,7 +1119,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>9</v>
@@ -1128,7 +1142,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>7</v>
@@ -1137,7 +1151,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>9</v>
@@ -1160,7 +1174,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>7</v>
@@ -1183,7 +1197,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>7</v>
@@ -1206,7 +1220,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B17" s="3">
         <v>9.525462962962963E-3</v>
@@ -1229,7 +1243,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>7</v>
@@ -1237,7 +1251,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>9</v>
@@ -1248,7 +1262,7 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>9</v>
@@ -1257,12 +1271,12 @@
         <v>7.5289351851851857E-2</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>9</v>
@@ -1273,15 +1287,15 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>9</v>
@@ -1292,7 +1306,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>9</v>
@@ -1303,7 +1317,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>9</v>
@@ -1318,12 +1332,12 @@
         <v>8</v>
       </c>
       <c r="H25" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B26" s="3">
         <v>1.8981481481481482E-3</v>
@@ -1334,7 +1348,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>9</v>
@@ -1345,7 +1359,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>9</v>
@@ -1356,7 +1370,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>9</v>
@@ -1367,7 +1381,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>9</v>
@@ -1378,7 +1392,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B31" s="3">
         <v>4.2013888888888891E-3</v>
@@ -1389,7 +1403,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B32" s="3">
         <v>8.8078703703703704E-3</v>
@@ -1400,7 +1414,7 @@
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>9</v>
@@ -1411,7 +1425,7 @@
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>9</v>
@@ -1422,7 +1436,7 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>9</v>
@@ -1433,7 +1447,7 @@
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>9</v>
@@ -1444,7 +1458,7 @@
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>9</v>
@@ -1455,7 +1469,7 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>9</v>
@@ -1466,7 +1480,7 @@
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>9</v>
@@ -1475,12 +1489,12 @@
         <v>8</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>9</v>
@@ -1498,12 +1512,12 @@
         <v>0.22163194444444445</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>7</v>
@@ -1511,7 +1525,7 @@
     </row>
     <row r="42" spans="1:7">
       <c r="A42" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>7</v>
@@ -1519,7 +1533,7 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>9</v>
@@ -1530,7 +1544,7 @@
     </row>
     <row r="44" spans="1:7">
       <c r="A44" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>10</v>
@@ -1538,7 +1552,7 @@
     </row>
     <row r="45" spans="1:7">
       <c r="A45" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>9</v>
@@ -1549,7 +1563,7 @@
     </row>
     <row r="46" spans="1:7">
       <c r="A46" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>9</v>
@@ -1560,7 +1574,7 @@
     </row>
     <row r="47" spans="1:7">
       <c r="A47" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>9</v>
@@ -1571,7 +1585,7 @@
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>9</v>
@@ -1582,7 +1596,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>10</v>
@@ -1590,7 +1604,7 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>9</v>
@@ -1601,7 +1615,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B51" s="3">
         <v>1.1238425925925926E-2</v>
@@ -1612,7 +1626,7 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>9</v>
@@ -1623,7 +1637,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>9</v>
@@ -1638,12 +1652,12 @@
         <v>0.19527777777777777</v>
       </c>
       <c r="H53" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>9</v>
@@ -1654,10 +1668,10 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C55" s="3">
         <v>9.6782407407407414E-2</v>
@@ -1665,7 +1679,7 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B56" s="3">
         <v>5.0694444444444441E-3</v>
@@ -1676,7 +1690,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>9</v>
@@ -1687,7 +1701,7 @@
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B58" s="3">
         <v>1.480324074074074E-2</v>
@@ -1698,7 +1712,7 @@
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>9</v>
@@ -1709,7 +1723,7 @@
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>9</v>
@@ -1720,198 +1734,369 @@
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" s="3">
+        <v>7.6087962962962968E-2</v>
       </c>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
+      </c>
+      <c r="B63" s="3">
+        <v>1.5949074074074074E-2</v>
+      </c>
+      <c r="C63" s="3">
+        <v>7.4652777777777776E-2</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B64" s="3">
+        <v>2.8935185185185184E-4</v>
+      </c>
+      <c r="C64" s="3">
+        <v>0.11217592592592593</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="65" spans="1:1">
-      <c r="A65" s="2" t="s">
+      <c r="B65" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C65" s="3">
+        <v>0.1973263888888889</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="66" spans="1:1">
-      <c r="A66" s="2" t="s">
+      <c r="B66" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="67" spans="1:1">
-      <c r="A67" s="2" t="s">
+      <c r="B67" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C67" s="3">
+        <v>8.9490740740740746E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="68" spans="1:1">
-      <c r="A68" s="2" t="s">
+      <c r="B68" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C68" s="3">
+        <v>7.0231481481481478E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="69" spans="1:1">
-      <c r="A69" s="2" t="s">
+      <c r="B69" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" s="3">
+        <v>7.4722222222222218E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="70" spans="1:1">
-      <c r="A70" s="2" t="s">
+      <c r="B70" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" s="3">
+        <v>6.322916666666667E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="71" spans="1:1">
-      <c r="A71" s="2" t="s">
+      <c r="B71" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" s="3">
+        <v>0.15739583333333335</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="72" spans="1:1">
-      <c r="A72" s="2" t="s">
+      <c r="B72" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C72" s="3">
+        <v>5.1446759259259262E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" s="2" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="73" spans="1:1">
-      <c r="A73" s="2" t="s">
+      <c r="B73" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C73" s="3">
+        <v>0.22515046296296296</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="74" spans="1:1">
-      <c r="A74" s="2" t="s">
+      <c r="B74" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C74" s="3">
+        <v>8.0057870370370376E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="75" spans="1:1">
-      <c r="A75" s="2" t="s">
+      <c r="B75" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C75" s="3">
+        <v>6.0011574074074071E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="76" spans="1:1">
-      <c r="A76" s="2" t="s">
+      <c r="B76" s="3">
+        <v>5.2662037037037035E-3</v>
+      </c>
+      <c r="C76" s="3">
+        <v>4.3090277777777776E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" s="2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="77" spans="1:1">
-      <c r="A77" s="2" t="s">
+      <c r="B77" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="78" spans="1:1">
-      <c r="A78" s="2" t="s">
+      <c r="B78" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" s="2" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="79" spans="1:1">
-      <c r="A79" s="2" t="s">
+      <c r="B79" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C79" s="3">
+        <v>0.27971064814814817</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="80" spans="1:1">
-      <c r="A80" s="2" t="s">
+      <c r="B80" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8">
+      <c r="A81" s="2" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="81" spans="1:7">
-      <c r="A81" s="2" t="s">
+      <c r="B81" s="3">
+        <v>2.150462962962963E-2</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8">
+      <c r="A82" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="82" spans="1:7">
-      <c r="A82" s="2" t="s">
+      <c r="B82" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8">
+      <c r="A83" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B82" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G82" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7">
-      <c r="A83" s="2" t="s">
+      <c r="B83" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C83" s="3">
+        <v>0.10276620370370371</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
+      <c r="A84" s="2" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="84" spans="1:7">
-      <c r="A84" s="2" t="s">
+      <c r="B84" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C84" s="3">
+        <v>0.12923611111111111</v>
+      </c>
+      <c r="D84" s="3">
+        <v>0.15792824074074074</v>
+      </c>
+      <c r="E84" s="3">
+        <v>0.21453703703703703</v>
+      </c>
+      <c r="H84" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="85" spans="1:7">
-      <c r="A85" s="2" t="s">
+      <c r="B85" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
+      <c r="A86" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E85" s="3">
+      <c r="B86" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C86" s="3">
         <v>6.0011574074074071E-2</v>
       </c>
-      <c r="F85" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G85" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7">
-      <c r="A86" s="2" t="s">
+    </row>
+    <row r="87" spans="1:8">
+      <c r="A87" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="87" spans="1:7">
-      <c r="A87" s="2" t="s">
+      <c r="B87" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8">
+      <c r="A88" s="2" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="88" spans="1:7">
-      <c r="A88" s="2" t="s">
+      <c r="B88" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C88" s="3">
+        <v>5.6423611111111112E-2</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H88" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8">
+      <c r="A89" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="89" spans="1:7">
-      <c r="A89" s="2" t="s">
+      <c r="B89" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
+      <c r="A90" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="90" spans="1:7">
-      <c r="A90" s="2" t="s">
+      <c r="B90" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C90" s="3">
+        <v>0.15649305555555557</v>
+      </c>
+      <c r="D90" s="3">
+        <v>0.19611111111111112</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8">
+      <c r="A91" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="91" spans="1:7">
-      <c r="A91" s="2" t="s">
+      <c r="B91" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C91" s="3">
+        <v>4.8865740740740737E-2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8">
+      <c r="A92" s="2" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7">
-      <c r="A92" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>9</v>
@@ -1923,7 +2108,7 @@
         <v>0.1102662037037037</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>7</v>
@@ -1932,24 +2117,42 @@
         <v>7</v>
       </c>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:8">
       <c r="A93" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8">
+      <c r="A94" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="94" spans="1:7">
-      <c r="A94" s="2" t="s">
+      <c r="B94" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8">
+      <c r="A95" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="95" spans="1:7">
-      <c r="A95" s="2" t="s">
+      <c r="B95" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C95" s="3">
+        <v>9.4502314814814817E-2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8">
+      <c r="A96" s="2" t="s">
         <v>107</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7">
-      <c r="A96" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>9</v>
@@ -1972,12 +2175,18 @@
     </row>
     <row r="97" spans="1:7">
       <c r="A97" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="98" spans="1:7">
       <c r="A98" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>9</v>
@@ -2000,17 +2209,29 @@
     </row>
     <row r="99" spans="1:7">
       <c r="A99" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="100" spans="1:7">
       <c r="A100" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C100" s="3">
+        <v>8.1215277777777775E-2</v>
       </c>
     </row>
     <row r="101" spans="1:7">
       <c r="A101" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>9</v>
@@ -2033,17 +2254,29 @@
     </row>
     <row r="102" spans="1:7">
       <c r="A102" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="103" spans="1:7">
       <c r="A103" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="104" spans="1:7">
       <c r="A104" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>9</v>
@@ -2066,22 +2299,40 @@
     </row>
     <row r="105" spans="1:7">
       <c r="A105" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="106" spans="1:7">
       <c r="A106" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C106" s="3">
+        <v>6.0798611111111109E-2</v>
       </c>
     </row>
     <row r="107" spans="1:7">
       <c r="A107" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C107" s="3">
+        <v>0.11762731481481481</v>
       </c>
     </row>
     <row r="108" spans="1:7">
       <c r="A108" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>9</v>
@@ -2104,30 +2355,54 @@
     </row>
     <row r="109" spans="1:7">
       <c r="A109" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="110" spans="1:7">
       <c r="A110" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
+      </c>
+      <c r="B110" s="3">
+        <v>1.0416666666666667E-4</v>
+      </c>
+      <c r="C110" s="3">
+        <v>0.16601851851851851</v>
       </c>
     </row>
     <row r="111" spans="1:7">
       <c r="A111" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C111" s="3">
+        <v>5.8495370370370371E-2</v>
       </c>
     </row>
     <row r="112" spans="1:7">
       <c r="A112" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C112" s="3">
+        <v>9.7256944444444438E-2</v>
       </c>
     </row>
     <row r="113" spans="1:7">
       <c r="A113" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C113" s="3">
         <v>3.9849537037037037E-2</v>
@@ -2136,7 +2411,7 @@
         <v>7.3969907407407401E-2</v>
       </c>
       <c r="E113" s="3">
-        <v>0.10035879629629629</v>
+        <v>0.10069444444444445</v>
       </c>
       <c r="F113" s="3">
         <v>0.12188657407407408</v>
@@ -2147,137 +2422,227 @@
     </row>
     <row r="114" spans="1:7">
       <c r="A114" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="115" spans="1:7">
       <c r="A115" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="116" spans="1:7">
       <c r="A116" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C116" s="3">
+        <v>0.17356481481481481</v>
       </c>
     </row>
     <row r="117" spans="1:7">
       <c r="A117" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="118" spans="1:7">
       <c r="A118" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="119" spans="1:7">
       <c r="A119" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="120" spans="1:7">
       <c r="A120" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D120" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E120" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F120" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G120" s="2" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
     </row>
     <row r="121" spans="1:7">
       <c r="A121" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="122" spans="1:7">
       <c r="A122" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="123" spans="1:7">
       <c r="A123" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="124" spans="1:7">
       <c r="A124" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="125" spans="1:7">
       <c r="A125" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D125" s="3">
+        <v>8.1180555555555561E-2</v>
+      </c>
+      <c r="E125" s="3">
+        <v>0.12420138888888889</v>
       </c>
     </row>
     <row r="126" spans="1:7">
       <c r="A126" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
+      </c>
+      <c r="B126" s="3">
+        <v>9.4907407407407408E-4</v>
+      </c>
+      <c r="C126" s="3">
+        <v>0.11008101851851852</v>
       </c>
     </row>
     <row r="127" spans="1:7">
       <c r="A127" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="128" spans="1:7">
       <c r="A128" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="129" spans="1:7">
       <c r="A129" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="130" spans="1:7">
       <c r="A130" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="131" spans="1:7">
       <c r="A131" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="132" spans="1:7">
       <c r="A132" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="133" spans="1:7">
       <c r="A133" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="134" spans="1:7">
       <c r="A134" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>9</v>
@@ -2300,171 +2665,327 @@
     </row>
     <row r="135" spans="1:7">
       <c r="A135" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="136" spans="1:7">
       <c r="A136" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C136" s="3">
+        <v>0.11761574074074074</v>
       </c>
     </row>
     <row r="137" spans="1:7">
       <c r="A137" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C137" s="3">
+        <v>9.0937500000000004E-2</v>
+      </c>
+      <c r="D137" s="3">
+        <v>0.12048611111111111</v>
+      </c>
+      <c r="E137" s="3">
+        <v>0.23645833333333333</v>
       </c>
     </row>
     <row r="138" spans="1:7">
       <c r="A138" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="139" spans="1:7">
       <c r="A139" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C139" s="3">
+        <v>3.9293981481481478E-2</v>
+      </c>
+      <c r="D139" s="3">
+        <v>8.9340277777777782E-2</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="140" spans="1:7">
       <c r="A140" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="141" spans="1:7">
       <c r="A141" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="142" spans="1:7">
       <c r="A142" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="143" spans="1:7">
       <c r="A143" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="144" spans="1:7">
       <c r="A144" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3">
+      <c r="A145" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="145" spans="1:2">
-      <c r="A145" s="2" t="s">
+      <c r="B145" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3">
+      <c r="A146" s="2" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="146" spans="1:2">
-      <c r="A146" s="2" t="s">
+      <c r="B146" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3">
+      <c r="A147" s="2" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="147" spans="1:2">
-      <c r="A147" s="2" t="s">
+      <c r="B147" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3">
+      <c r="A148" s="2" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="148" spans="1:2">
-      <c r="A148" s="2" t="s">
+      <c r="B148" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3">
+      <c r="A149" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="149" spans="1:2">
-      <c r="A149" s="2" t="s">
+      <c r="B149" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3">
+      <c r="A150" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B149" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2">
-      <c r="A150" s="2" t="s">
+      <c r="B150" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3">
+      <c r="A151" s="2" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="151" spans="1:2">
-      <c r="A151" s="2" t="s">
+      <c r="B151" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3">
+      <c r="A152" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="152" spans="1:2">
-      <c r="A152" s="2" t="s">
+      <c r="B152" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3">
+      <c r="A153" s="2" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="153" spans="1:2">
-      <c r="A153" s="2" t="s">
+      <c r="B153" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3">
+      <c r="A154" s="2" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="154" spans="1:2">
-      <c r="A154" s="2" t="s">
+      <c r="B154" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3">
+      <c r="A155" s="2" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="155" spans="1:2">
-      <c r="A155" s="2" t="s">
+      <c r="B155" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3">
+      <c r="A156" s="2" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="156" spans="1:2">
-      <c r="A156" s="2" t="s">
+      <c r="B156" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3">
+      <c r="A157" s="2" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="157" spans="1:2">
-      <c r="A157" s="2" t="s">
+      <c r="B157" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3">
+      <c r="A158" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B157" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2">
-      <c r="A158" s="2" t="s">
+      <c r="B158" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3">
+      <c r="A159" s="2" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="159" spans="1:2">
-      <c r="A159" s="2" t="s">
+      <c r="B159" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3">
+      <c r="A160" s="2" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="160" spans="1:2">
-      <c r="A160" s="2" t="s">
+      <c r="B160" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8">
+      <c r="A161" s="2" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="161" spans="1:7">
-      <c r="A161" s="2" t="s">
+      <c r="B161" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8">
+      <c r="A162" s="2" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="162" spans="1:7">
-      <c r="A162" s="2" t="s">
+      <c r="B162" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8">
+      <c r="A163" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B162" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7">
-      <c r="A163" s="2" t="s">
+      <c r="B163" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8">
+      <c r="A164" s="2" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="164" spans="1:7">
-      <c r="A164" s="2" t="s">
+      <c r="B164" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8">
+      <c r="A165" s="2" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="165" spans="1:7">
-      <c r="A165" s="2" t="s">
+      <c r="B165" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8">
+      <c r="A166" s="2" t="s">
         <v>177</v>
-      </c>
-    </row>
-    <row r="166" spans="1:7">
-      <c r="A166" s="2" t="s">
-        <v>178</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>9</v>
@@ -2485,24 +3006,42 @@
         <v>0.26956018518518521</v>
       </c>
     </row>
-    <row r="167" spans="1:7">
+    <row r="167" spans="1:8">
       <c r="A167" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8">
+      <c r="A168" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="168" spans="1:7">
-      <c r="A168" s="2" t="s">
+      <c r="B168" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8">
+      <c r="A169" s="2" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="169" spans="1:7">
-      <c r="A169" s="2" t="s">
+      <c r="B169" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C169" s="3">
+        <v>0.14844907407407407</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8">
+      <c r="A170" s="2" t="s">
         <v>181</v>
-      </c>
-    </row>
-    <row r="170" spans="1:7">
-      <c r="A170" s="2" t="s">
-        <v>182</v>
       </c>
       <c r="B170" s="3">
         <v>5.37037037037037E-3</v>
@@ -2522,40 +3061,85 @@
       <c r="G170" s="3">
         <v>0.26238425925925923</v>
       </c>
-    </row>
-    <row r="171" spans="1:7">
+      <c r="H170" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8">
       <c r="A171" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B171" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8">
+      <c r="A172" s="2" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="172" spans="1:7">
-      <c r="A172" s="2" t="s">
+      <c r="B172" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C172" s="3">
+        <v>0.10276620370370371</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8">
+      <c r="A173" s="2" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="173" spans="1:7">
-      <c r="A173" s="2" t="s">
+      <c r="B173" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C173" s="3">
+        <v>0.1575</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8">
+      <c r="A174" s="2" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="174" spans="1:7">
-      <c r="A174" s="2" t="s">
+      <c r="B174" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C174" s="3">
+        <v>0.17703703703703705</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8">
+      <c r="A175" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="175" spans="1:7">
-      <c r="A175" s="2" t="s">
+      <c r="B175" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C175" s="3">
+        <v>9.268518518518519E-2</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8">
+      <c r="A176" s="2" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="176" spans="1:7">
-      <c r="A176" s="2" t="s">
+      <c r="B176" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3">
+      <c r="A177" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="177" spans="1:1">
-      <c r="A177" s="2" t="s">
-        <v>189</v>
+      <c r="B177" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C177" s="3">
+        <v>0.18931712962962963</v>
       </c>
     </row>
     <row r="239" spans="1:1">

</xml_diff>

<commit_message>
on lab- finish update times .xlsx
</commit_message>
<xml_diff>
--- a/times .xlsx
+++ b/times .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Room_8_Data\Scalpel_Raz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDEB2F3-8FDF-4D85-A515-D5E7FDCAA80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6755F6-9E17-48AE-95AF-D7B8A2C65CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="201">
   <si>
     <t>date</t>
   </si>
@@ -63,9 +63,6 @@
     <t>?</t>
   </si>
   <si>
-    <t>prbably end</t>
-  </si>
-  <si>
     <t>v</t>
   </si>
   <si>
@@ -613,6 +610,24 @@
   </si>
   <si>
     <t xml:space="preserve"> start</t>
+  </si>
+  <si>
+    <t>very long</t>
+  </si>
+  <si>
+    <t>14hrs</t>
+  </si>
+  <si>
+    <t>50hr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  01:13:07</t>
+  </si>
+  <si>
+    <t>19hr</t>
+  </si>
+  <si>
+    <t>Foramt problem. Export again</t>
   </si>
 </sst>
 </file>
@@ -985,8 +1000,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="45.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="19.125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="39.5" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.75" style="2" customWidth="1"/>
     <col min="6" max="6" width="16.5" style="2" bestFit="1" customWidth="1"/>
@@ -1019,15 +1033,15 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>7</v>
@@ -1035,7 +1049,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>7</v>
@@ -1043,26 +1057,26 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
@@ -1070,7 +1084,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>7</v>
@@ -1078,23 +1092,23 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>9</v>
@@ -1105,7 +1119,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>9</v>
@@ -1128,7 +1142,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>7</v>
@@ -1137,7 +1151,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>9</v>
@@ -1160,7 +1174,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>7</v>
@@ -1183,7 +1197,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>7</v>
@@ -1206,7 +1220,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B17" s="3">
         <v>9.525462962962963E-3</v>
@@ -1229,7 +1243,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>7</v>
@@ -1237,7 +1251,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>9</v>
@@ -1248,7 +1262,7 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>9</v>
@@ -1257,12 +1271,12 @@
         <v>7.5289351851851857E-2</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>9</v>
@@ -1273,15 +1287,15 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>9</v>
@@ -1292,7 +1306,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>9</v>
@@ -1303,7 +1317,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>9</v>
@@ -1318,12 +1332,12 @@
         <v>8</v>
       </c>
       <c r="H25" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B26" s="3">
         <v>1.8981481481481482E-3</v>
@@ -1334,7 +1348,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>9</v>
@@ -1345,7 +1359,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>9</v>
@@ -1356,7 +1370,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>9</v>
@@ -1367,7 +1381,7 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>9</v>
@@ -1378,7 +1392,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B31" s="3">
         <v>4.2013888888888891E-3</v>
@@ -1389,7 +1403,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B32" s="3">
         <v>8.8078703703703704E-3</v>
@@ -1400,7 +1414,7 @@
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>9</v>
@@ -1411,7 +1425,7 @@
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>9</v>
@@ -1422,7 +1436,7 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>9</v>
@@ -1433,7 +1447,7 @@
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>9</v>
@@ -1444,7 +1458,7 @@
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>9</v>
@@ -1455,7 +1469,7 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>9</v>
@@ -1466,7 +1480,7 @@
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>9</v>
@@ -1475,12 +1489,12 @@
         <v>8</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>9</v>
@@ -1498,12 +1512,12 @@
         <v>0.22163194444444445</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>7</v>
@@ -1511,7 +1525,7 @@
     </row>
     <row r="42" spans="1:7">
       <c r="A42" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>7</v>
@@ -1519,7 +1533,7 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>9</v>
@@ -1530,7 +1544,7 @@
     </row>
     <row r="44" spans="1:7">
       <c r="A44" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>10</v>
@@ -1538,7 +1552,7 @@
     </row>
     <row r="45" spans="1:7">
       <c r="A45" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>9</v>
@@ -1549,7 +1563,7 @@
     </row>
     <row r="46" spans="1:7">
       <c r="A46" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>9</v>
@@ -1560,7 +1574,7 @@
     </row>
     <row r="47" spans="1:7">
       <c r="A47" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>9</v>
@@ -1571,7 +1585,7 @@
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>9</v>
@@ -1582,7 +1596,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>10</v>
@@ -1590,7 +1604,7 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>9</v>
@@ -1601,7 +1615,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B51" s="3">
         <v>1.1238425925925926E-2</v>
@@ -1612,7 +1626,7 @@
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>9</v>
@@ -1623,7 +1637,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>9</v>
@@ -1638,12 +1652,12 @@
         <v>0.19527777777777777</v>
       </c>
       <c r="H53" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>9</v>
@@ -1654,10 +1668,10 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C55" s="3">
         <v>9.6782407407407414E-2</v>
@@ -1665,7 +1679,7 @@
     </row>
     <row r="56" spans="1:8">
       <c r="A56" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B56" s="3">
         <v>5.0694444444444441E-3</v>
@@ -1676,7 +1690,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>9</v>
@@ -1687,7 +1701,7 @@
     </row>
     <row r="58" spans="1:8">
       <c r="A58" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B58" s="3">
         <v>1.480324074074074E-2</v>
@@ -1698,7 +1712,7 @@
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>9</v>
@@ -1709,7 +1723,7 @@
     </row>
     <row r="60" spans="1:8">
       <c r="A60" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>9</v>
@@ -1720,198 +1734,369 @@
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" s="3">
+        <v>7.6087962962962968E-2</v>
       </c>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
+      </c>
+      <c r="B63" s="3">
+        <v>1.5949074074074074E-2</v>
+      </c>
+      <c r="C63" s="3">
+        <v>7.4652777777777776E-2</v>
       </c>
     </row>
     <row r="64" spans="1:8">
       <c r="A64" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B64" s="3">
+        <v>2.8935185185185184E-4</v>
+      </c>
+      <c r="C64" s="3">
+        <v>0.11217592592592593</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="65" spans="1:1">
-      <c r="A65" s="2" t="s">
+      <c r="B65" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C65" s="3">
+        <v>0.1973263888888889</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="66" spans="1:1">
-      <c r="A66" s="2" t="s">
+      <c r="B66" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="67" spans="1:1">
-      <c r="A67" s="2" t="s">
+      <c r="B67" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C67" s="3">
+        <v>8.9490740740740746E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="68" spans="1:1">
-      <c r="A68" s="2" t="s">
+      <c r="B68" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C68" s="3">
+        <v>7.0231481481481478E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="69" spans="1:1">
-      <c r="A69" s="2" t="s">
+      <c r="B69" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" s="3">
+        <v>7.4722222222222218E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="70" spans="1:1">
-      <c r="A70" s="2" t="s">
+      <c r="B70" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" s="3">
+        <v>6.322916666666667E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="71" spans="1:1">
-      <c r="A71" s="2" t="s">
+      <c r="B71" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" s="3">
+        <v>0.15739583333333335</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="72" spans="1:1">
-      <c r="A72" s="2" t="s">
+      <c r="B72" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C72" s="3">
+        <v>5.1446759259259262E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" s="2" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="73" spans="1:1">
-      <c r="A73" s="2" t="s">
+      <c r="B73" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C73" s="3">
+        <v>0.22515046296296296</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="74" spans="1:1">
-      <c r="A74" s="2" t="s">
+      <c r="B74" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C74" s="3">
+        <v>8.0057870370370376E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="75" spans="1:1">
-      <c r="A75" s="2" t="s">
+      <c r="B75" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C75" s="3">
+        <v>6.0011574074074071E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="76" spans="1:1">
-      <c r="A76" s="2" t="s">
+      <c r="B76" s="3">
+        <v>5.2662037037037035E-3</v>
+      </c>
+      <c r="C76" s="3">
+        <v>4.3090277777777776E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" s="2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="77" spans="1:1">
-      <c r="A77" s="2" t="s">
+      <c r="B77" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="78" spans="1:1">
-      <c r="A78" s="2" t="s">
+      <c r="B78" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" s="2" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="79" spans="1:1">
-      <c r="A79" s="2" t="s">
+      <c r="B79" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C79" s="3">
+        <v>0.27971064814814817</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="80" spans="1:1">
-      <c r="A80" s="2" t="s">
+      <c r="B80" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8">
+      <c r="A81" s="2" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="81" spans="1:7">
-      <c r="A81" s="2" t="s">
+      <c r="B81" s="3">
+        <v>2.150462962962963E-2</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8">
+      <c r="A82" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="82" spans="1:7">
-      <c r="A82" s="2" t="s">
+      <c r="B82" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8">
+      <c r="A83" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B82" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G82" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7">
-      <c r="A83" s="2" t="s">
+      <c r="B83" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C83" s="3">
+        <v>0.10276620370370371</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
+      <c r="A84" s="2" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="84" spans="1:7">
-      <c r="A84" s="2" t="s">
+      <c r="B84" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C84" s="3">
+        <v>0.12923611111111111</v>
+      </c>
+      <c r="D84" s="3">
+        <v>0.15792824074074074</v>
+      </c>
+      <c r="E84" s="3">
+        <v>0.21453703703703703</v>
+      </c>
+      <c r="H84" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="85" spans="1:7">
-      <c r="A85" s="2" t="s">
+      <c r="B85" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
+      <c r="A86" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E85" s="3">
+      <c r="B86" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C86" s="3">
         <v>6.0011574074074071E-2</v>
       </c>
-      <c r="F85" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G85" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7">
-      <c r="A86" s="2" t="s">
+    </row>
+    <row r="87" spans="1:8">
+      <c r="A87" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="87" spans="1:7">
-      <c r="A87" s="2" t="s">
+      <c r="B87" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8">
+      <c r="A88" s="2" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="88" spans="1:7">
-      <c r="A88" s="2" t="s">
+      <c r="B88" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C88" s="3">
+        <v>5.6423611111111112E-2</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H88" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8">
+      <c r="A89" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="89" spans="1:7">
-      <c r="A89" s="2" t="s">
+      <c r="B89" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
+      <c r="A90" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="90" spans="1:7">
-      <c r="A90" s="2" t="s">
+      <c r="B90" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C90" s="3">
+        <v>0.15649305555555557</v>
+      </c>
+      <c r="D90" s="3">
+        <v>0.19611111111111112</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8">
+      <c r="A91" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="91" spans="1:7">
-      <c r="A91" s="2" t="s">
+      <c r="B91" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C91" s="3">
+        <v>4.8865740740740737E-2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8">
+      <c r="A92" s="2" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7">
-      <c r="A92" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>9</v>
@@ -1923,7 +2108,7 @@
         <v>0.1102662037037037</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>7</v>
@@ -1932,24 +2117,42 @@
         <v>7</v>
       </c>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:8">
       <c r="A93" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8">
+      <c r="A94" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="94" spans="1:7">
-      <c r="A94" s="2" t="s">
+      <c r="B94" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8">
+      <c r="A95" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="95" spans="1:7">
-      <c r="A95" s="2" t="s">
+      <c r="B95" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C95" s="3">
+        <v>9.4502314814814817E-2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8">
+      <c r="A96" s="2" t="s">
         <v>107</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7">
-      <c r="A96" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>9</v>
@@ -1972,12 +2175,18 @@
     </row>
     <row r="97" spans="1:7">
       <c r="A97" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="98" spans="1:7">
       <c r="A98" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>9</v>
@@ -2000,17 +2209,29 @@
     </row>
     <row r="99" spans="1:7">
       <c r="A99" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="100" spans="1:7">
       <c r="A100" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C100" s="3">
+        <v>8.1215277777777775E-2</v>
       </c>
     </row>
     <row r="101" spans="1:7">
       <c r="A101" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>9</v>
@@ -2033,17 +2254,29 @@
     </row>
     <row r="102" spans="1:7">
       <c r="A102" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="103" spans="1:7">
       <c r="A103" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="104" spans="1:7">
       <c r="A104" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>9</v>
@@ -2066,22 +2299,40 @@
     </row>
     <row r="105" spans="1:7">
       <c r="A105" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="106" spans="1:7">
       <c r="A106" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C106" s="3">
+        <v>6.0798611111111109E-2</v>
       </c>
     </row>
     <row r="107" spans="1:7">
       <c r="A107" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C107" s="3">
+        <v>0.11762731481481481</v>
       </c>
     </row>
     <row r="108" spans="1:7">
       <c r="A108" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>9</v>
@@ -2104,30 +2355,54 @@
     </row>
     <row r="109" spans="1:7">
       <c r="A109" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="110" spans="1:7">
       <c r="A110" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
+      </c>
+      <c r="B110" s="3">
+        <v>1.0416666666666667E-4</v>
+      </c>
+      <c r="C110" s="3">
+        <v>0.16601851851851851</v>
       </c>
     </row>
     <row r="111" spans="1:7">
       <c r="A111" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C111" s="3">
+        <v>5.8495370370370371E-2</v>
       </c>
     </row>
     <row r="112" spans="1:7">
       <c r="A112" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C112" s="3">
+        <v>9.7256944444444438E-2</v>
       </c>
     </row>
     <row r="113" spans="1:7">
       <c r="A113" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C113" s="3">
         <v>3.9849537037037037E-2</v>
@@ -2136,7 +2411,7 @@
         <v>7.3969907407407401E-2</v>
       </c>
       <c r="E113" s="3">
-        <v>0.10035879629629629</v>
+        <v>0.10069444444444445</v>
       </c>
       <c r="F113" s="3">
         <v>0.12188657407407408</v>
@@ -2147,137 +2422,227 @@
     </row>
     <row r="114" spans="1:7">
       <c r="A114" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="115" spans="1:7">
       <c r="A115" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="116" spans="1:7">
       <c r="A116" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C116" s="3">
+        <v>0.17356481481481481</v>
       </c>
     </row>
     <row r="117" spans="1:7">
       <c r="A117" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="118" spans="1:7">
       <c r="A118" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="119" spans="1:7">
       <c r="A119" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="120" spans="1:7">
       <c r="A120" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D120" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E120" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F120" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G120" s="2" t="s">
-        <v>11</v>
+        <v>189</v>
       </c>
     </row>
     <row r="121" spans="1:7">
       <c r="A121" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="122" spans="1:7">
       <c r="A122" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="123" spans="1:7">
       <c r="A123" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="124" spans="1:7">
       <c r="A124" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="125" spans="1:7">
       <c r="A125" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D125" s="3">
+        <v>8.1180555555555561E-2</v>
+      </c>
+      <c r="E125" s="3">
+        <v>0.12420138888888889</v>
       </c>
     </row>
     <row r="126" spans="1:7">
       <c r="A126" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
+      </c>
+      <c r="B126" s="3">
+        <v>9.4907407407407408E-4</v>
+      </c>
+      <c r="C126" s="3">
+        <v>0.11008101851851852</v>
       </c>
     </row>
     <row r="127" spans="1:7">
       <c r="A127" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="128" spans="1:7">
       <c r="A128" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="129" spans="1:7">
       <c r="A129" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="130" spans="1:7">
       <c r="A130" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="131" spans="1:7">
       <c r="A131" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="132" spans="1:7">
       <c r="A132" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="133" spans="1:7">
       <c r="A133" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="134" spans="1:7">
       <c r="A134" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>9</v>
@@ -2300,171 +2665,327 @@
     </row>
     <row r="135" spans="1:7">
       <c r="A135" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="136" spans="1:7">
       <c r="A136" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C136" s="3">
+        <v>0.11761574074074074</v>
       </c>
     </row>
     <row r="137" spans="1:7">
       <c r="A137" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C137" s="3">
+        <v>9.0937500000000004E-2</v>
+      </c>
+      <c r="D137" s="3">
+        <v>0.12048611111111111</v>
+      </c>
+      <c r="E137" s="3">
+        <v>0.23645833333333333</v>
       </c>
     </row>
     <row r="138" spans="1:7">
       <c r="A138" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="139" spans="1:7">
       <c r="A139" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C139" s="3">
+        <v>3.9293981481481478E-2</v>
+      </c>
+      <c r="D139" s="3">
+        <v>8.9340277777777782E-2</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="140" spans="1:7">
       <c r="A140" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="141" spans="1:7">
       <c r="A141" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="142" spans="1:7">
       <c r="A142" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="143" spans="1:7">
       <c r="A143" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="144" spans="1:7">
       <c r="A144" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3">
+      <c r="A145" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="145" spans="1:2">
-      <c r="A145" s="2" t="s">
+      <c r="B145" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3">
+      <c r="A146" s="2" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="146" spans="1:2">
-      <c r="A146" s="2" t="s">
+      <c r="B146" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3">
+      <c r="A147" s="2" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="147" spans="1:2">
-      <c r="A147" s="2" t="s">
+      <c r="B147" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3">
+      <c r="A148" s="2" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="148" spans="1:2">
-      <c r="A148" s="2" t="s">
+      <c r="B148" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3">
+      <c r="A149" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="149" spans="1:2">
-      <c r="A149" s="2" t="s">
+      <c r="B149" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3">
+      <c r="A150" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B149" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2">
-      <c r="A150" s="2" t="s">
+      <c r="B150" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3">
+      <c r="A151" s="2" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="151" spans="1:2">
-      <c r="A151" s="2" t="s">
+      <c r="B151" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3">
+      <c r="A152" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="152" spans="1:2">
-      <c r="A152" s="2" t="s">
+      <c r="B152" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3">
+      <c r="A153" s="2" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="153" spans="1:2">
-      <c r="A153" s="2" t="s">
+      <c r="B153" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3">
+      <c r="A154" s="2" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="154" spans="1:2">
-      <c r="A154" s="2" t="s">
+      <c r="B154" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3">
+      <c r="A155" s="2" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="155" spans="1:2">
-      <c r="A155" s="2" t="s">
+      <c r="B155" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3">
+      <c r="A156" s="2" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="156" spans="1:2">
-      <c r="A156" s="2" t="s">
+      <c r="B156" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3">
+      <c r="A157" s="2" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="157" spans="1:2">
-      <c r="A157" s="2" t="s">
+      <c r="B157" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3">
+      <c r="A158" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B157" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2">
-      <c r="A158" s="2" t="s">
+      <c r="B158" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3">
+      <c r="A159" s="2" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="159" spans="1:2">
-      <c r="A159" s="2" t="s">
+      <c r="B159" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3">
+      <c r="A160" s="2" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="160" spans="1:2">
-      <c r="A160" s="2" t="s">
+      <c r="B160" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8">
+      <c r="A161" s="2" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="161" spans="1:7">
-      <c r="A161" s="2" t="s">
+      <c r="B161" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8">
+      <c r="A162" s="2" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="162" spans="1:7">
-      <c r="A162" s="2" t="s">
+      <c r="B162" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8">
+      <c r="A163" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B162" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7">
-      <c r="A163" s="2" t="s">
+      <c r="B163" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8">
+      <c r="A164" s="2" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="164" spans="1:7">
-      <c r="A164" s="2" t="s">
+      <c r="B164" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8">
+      <c r="A165" s="2" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="165" spans="1:7">
-      <c r="A165" s="2" t="s">
+      <c r="B165" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8">
+      <c r="A166" s="2" t="s">
         <v>177</v>
-      </c>
-    </row>
-    <row r="166" spans="1:7">
-      <c r="A166" s="2" t="s">
-        <v>178</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>9</v>
@@ -2485,24 +3006,42 @@
         <v>0.26956018518518521</v>
       </c>
     </row>
-    <row r="167" spans="1:7">
+    <row r="167" spans="1:8">
       <c r="A167" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8">
+      <c r="A168" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="168" spans="1:7">
-      <c r="A168" s="2" t="s">
+      <c r="B168" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8">
+      <c r="A169" s="2" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="169" spans="1:7">
-      <c r="A169" s="2" t="s">
+      <c r="B169" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C169" s="3">
+        <v>0.14844907407407407</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8">
+      <c r="A170" s="2" t="s">
         <v>181</v>
-      </c>
-    </row>
-    <row r="170" spans="1:7">
-      <c r="A170" s="2" t="s">
-        <v>182</v>
       </c>
       <c r="B170" s="3">
         <v>5.37037037037037E-3</v>
@@ -2522,40 +3061,85 @@
       <c r="G170" s="3">
         <v>0.26238425925925923</v>
       </c>
-    </row>
-    <row r="171" spans="1:7">
+      <c r="H170" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8">
       <c r="A171" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B171" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8">
+      <c r="A172" s="2" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="172" spans="1:7">
-      <c r="A172" s="2" t="s">
+      <c r="B172" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C172" s="3">
+        <v>0.10276620370370371</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8">
+      <c r="A173" s="2" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="173" spans="1:7">
-      <c r="A173" s="2" t="s">
+      <c r="B173" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C173" s="3">
+        <v>0.1575</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8">
+      <c r="A174" s="2" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="174" spans="1:7">
-      <c r="A174" s="2" t="s">
+      <c r="B174" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C174" s="3">
+        <v>0.17703703703703705</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8">
+      <c r="A175" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="175" spans="1:7">
-      <c r="A175" s="2" t="s">
+      <c r="B175" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C175" s="3">
+        <v>9.268518518518519E-2</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8">
+      <c r="A176" s="2" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="176" spans="1:7">
-      <c r="A176" s="2" t="s">
+      <c r="B176" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3">
+      <c r="A177" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="177" spans="1:1">
-      <c r="A177" s="2" t="s">
-        <v>189</v>
+      <c r="B177" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C177" s="3">
+        <v>0.18931712962962963</v>
       </c>
     </row>
     <row r="239" spans="1:1">

</xml_diff>